<commit_message>
removed flagged from graphs
</commit_message>
<xml_diff>
--- a/data/results/larva_batch_summary.xlsx
+++ b/data/results/larva_batch_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T17"/>
+  <dimension ref="A1:T18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1586,6 +1586,74 @@
       </c>
       <c r="T17" t="inlineStr"/>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>..\data\csvs\N3_nSybxRalRNAi_L2_FA.csv</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>5402</v>
+      </c>
+      <c r="C18" t="n">
+        <v>27.78600518326546</v>
+      </c>
+      <c r="D18" t="n">
+        <v>50.03333333333333</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
+        <v>72.04662166194157</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0.5542047820149353</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.4242640687118441</v>
+      </c>
+      <c r="K18" t="n">
+        <v>3.012573650552031</v>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>N3</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>nSybxRalRNAi</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>FA</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="n">
+        <v>0.007021853179890999</v>
+      </c>
+      <c r="R18" t="n">
+        <v>0</v>
+      </c>
+      <c r="S18" t="b">
+        <v>0</v>
+      </c>
+      <c r="T18" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Group larvae analysis strictly by genotype and cohort folders, sanitize plot labels and improve figure layout
</commit_message>
<xml_diff>
--- a/data/results/larva_batch_summary.xlsx
+++ b/data/results/larva_batch_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T18"/>
+  <dimension ref="A1:T37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -521,7 +521,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>..\data\csvs\N1_nSybxRalRNAiBL29580_29C_L1_FA.csv</t>
+          <t>..\data\csvs\genotiponovo\N1\N1_nSybxRalRNAiBL29580_29C_L1_FA.csv</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -561,7 +561,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>nSybxRalRNAiBL29580</t>
+          <t>genotiponovo</t>
         </is>
       </c>
       <c r="N2" t="inlineStr"/>
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>..\data\csvs\N1_nSybxRalRNAiBL29580_29C_L2_FA.csv</t>
+          <t>..\data\csvs\genotiponovo\N1\N1_nSybxRalRNAiBL29580_29C_L2_FA.csv</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -625,7 +625,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>nSybxRalRNAiBL29580</t>
+          <t>genotiponovo</t>
         </is>
       </c>
       <c r="N3" t="inlineStr"/>
@@ -649,7 +649,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>..\data\csvs\N1_nSybxRalRNAiBL29580_29C_L3_FA.csv</t>
+          <t>..\data\csvs\genotiponovo\N1\N1_nSybxRalRNAiBL29580_29C_L3_FA.csv</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -689,7 +689,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>nSybxRalRNAiBL29580</t>
+          <t>genotiponovo</t>
         </is>
       </c>
       <c r="N4" t="inlineStr"/>
@@ -713,7 +713,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>..\data\csvs\N1_nSybxRalRNAiBL29580_29C_L4_FA.csv</t>
+          <t>..\data\csvs\genotiponovo\N1\N1_nSybxRalRNAiBL29580_29C_L4_FA.csv</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -753,7 +753,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>nSybxRalRNAiBL29580</t>
+          <t>genotiponovo</t>
         </is>
       </c>
       <c r="N5" t="inlineStr"/>
@@ -777,7 +777,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>..\data\csvs\N1_nSybxRalRNAiBL29580_29C_L5_FA.csv</t>
+          <t>..\data\csvs\genotiponovo\N1\N1_nSybxRalRNAiBL29580_29C_L5_FA.csv</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -817,7 +817,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>nSybxRalRNAiBL29580</t>
+          <t>genotiponovo</t>
         </is>
       </c>
       <c r="N6" t="inlineStr"/>
@@ -841,7 +841,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>..\data\csvs\N1_nSybxRalRNAiBL29580_29C_L6_FA.csv</t>
+          <t>..\data\csvs\genotiponovo\N1\N1_nSybxRalRNAiBL29580_29C_L6_FA.csv</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -881,7 +881,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>nSybxRalRNAiBL29580</t>
+          <t>genotiponovo</t>
         </is>
       </c>
       <c r="N7" t="inlineStr"/>
@@ -905,7 +905,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>..\data\csvs\N2_nSybxRalRNAi_L1_FA.csv</t>
+          <t>..\data\csvs\genotiponovo\N2\N2_nSybxRalRNAi_L1_FA.csv</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -945,7 +945,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>nSybxRalRNAi</t>
+          <t>genotiponovo</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -973,7 +973,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>..\data\csvs\N2_nSybxRalRNAi_L2_FA.csv</t>
+          <t>..\data\csvs\genotiponovo\N2\N2_nSybxRalRNAi_L2_FA.csv</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -1013,7 +1013,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>nSybxRalRNAi</t>
+          <t>genotiponovo</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1045,7 +1045,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>..\data\csvs\N2_nSybxRalRNAi_L3_FA.csv</t>
+          <t>..\data\csvs\genotiponovo\N2\N2_nSybxRalRNAi_L3_FA.csv</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -1085,7 +1085,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>nSybxRalRNAi</t>
+          <t>genotiponovo</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1113,7 +1113,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>..\data\csvs\N2_nSybxRalRNAi_L4_FA.csv</t>
+          <t>..\data\csvs\genotiponovo\N2\N2_nSybxRalRNAi_L4_FA.csv</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -1153,7 +1153,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>nSybxRalRNAi</t>
+          <t>genotiponovo</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1181,7 +1181,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>..\data\csvs\N2_nSybxRalRNAi_L5_FA.csv</t>
+          <t>..\data\csvs\genotiponovo\N2\N2_nSybxRalRNAi_L5_FA.csv</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -1221,7 +1221,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>nSybxRalRNAi</t>
+          <t>genotiponovo</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1249,7 +1249,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>..\data\csvs\N2_nSybxRalRNAi_L6_FA.csv</t>
+          <t>..\data\csvs\genotiponovo\N2\N2_nSybxRalRNAi_L6_FA.csv</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1289,7 +1289,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>nSybxRalRNAi</t>
+          <t>genotiponovo</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1317,7 +1317,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>..\data\csvs\N2_nSybxRalRNAi_L7_FA.csv</t>
+          <t>..\data\csvs\genotiponovo\N2\N2_nSybxRalRNAi_L7_FA.csv</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -1357,7 +1357,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>nSybxRalRNAi</t>
+          <t>genotiponovo</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1385,7 +1385,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>..\data\csvs\N2_nSybxRalRNAi_L8_FA.csv</t>
+          <t>..\data\csvs\genotiponovo\N2\N2_nSybxRalRNAi_L8_FA.csv</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1425,7 +1425,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>nSybxRalRNAi</t>
+          <t>genotiponovo</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1453,7 +1453,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>..\data\csvs\N2_nSybxRalRNAi_L9_FA.csv</t>
+          <t>..\data\csvs\genotiponovo\N2\N2_nSybxRalRNAi_L9_FA.csv</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>nSybxRalRNAi</t>
+          <t>genotiponovo</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1521,7 +1521,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>..\data\csvs\N3_nSybxRalRNAi_L1_FA.csv</t>
+          <t>..\data\csvs\genotiponovo\N3\N3_nSybxRalRNAi_L1_FA.csv</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1561,7 +1561,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>nSybxRalRNAi</t>
+          <t>genotiponovo</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1589,7 +1589,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>..\data\csvs\N3_nSybxRalRNAi_L2_FA.csv</t>
+          <t>..\data\csvs\genotiponovo\N3\N3_nSybxRalRNAi_L2_FA.csv</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>nSybxRalRNAi</t>
+          <t>genotiponovo</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1653,6 +1653,1278 @@
         <v>0</v>
       </c>
       <c r="T18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>..\data\csvs\genotiponovo\N3\N3_nSybxRalRNAi_L3_FA.csv</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>5402</v>
+      </c>
+      <c r="C19" t="n">
+        <v>38.68937430581266</v>
+      </c>
+      <c r="D19" t="n">
+        <v>52.16666666666666</v>
+      </c>
+      <c r="E19" t="n">
+        <v>43</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
+        <v>68.68420079634333</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0.6227035430312178</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.4459820624195625</v>
+      </c>
+      <c r="K19" t="n">
+        <v>3.947708195903186</v>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>N3</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>genotiponovo</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>FA</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="n">
+        <v>0.004965200000023708</v>
+      </c>
+      <c r="R19" t="n">
+        <v>0</v>
+      </c>
+      <c r="S19" t="b">
+        <v>0</v>
+      </c>
+      <c r="T19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>..\data\csvs\nSybxRalRNAi\N1\N1_nSybxRalRNAiBL29580_29C_L1_FA.csv</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>5402</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="n">
+        <v>113.9853976782455</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0.6331349621083807</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.5028916384273823</v>
+      </c>
+      <c r="K20" t="n">
+        <v>3.760664834839667</v>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>N1</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>nSybxRalRNAi</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>29C_L1_FA</t>
+        </is>
+      </c>
+      <c r="Q20" t="n">
+        <v>0.008951141596470501</v>
+      </c>
+      <c r="R20" t="n">
+        <v>0</v>
+      </c>
+      <c r="S20" t="b">
+        <v>0</v>
+      </c>
+      <c r="T20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>..\data\csvs\nSybxRalRNAi\N1\N1_nSybxRalRNAiBL29580_29C_L2_FA.csv</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>5403</v>
+      </c>
+      <c r="C21" t="n">
+        <v>76.73514714047751</v>
+      </c>
+      <c r="D21" t="n">
+        <v>81.8</v>
+      </c>
+      <c r="E21" t="n">
+        <v>72</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="n">
+        <v>53.79191090480974</v>
+      </c>
+      <c r="I21" t="n">
+        <v>1.289973882609346</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0.9904544411531474</v>
+      </c>
+      <c r="K21" t="n">
+        <v>5.589105474044938</v>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>N1</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>nSybxRalRNAi</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>29C_L2_FA</t>
+        </is>
+      </c>
+      <c r="Q21" t="n">
+        <v>0.004965200000006068</v>
+      </c>
+      <c r="R21" t="n">
+        <v>0</v>
+      </c>
+      <c r="S21" t="b">
+        <v>0</v>
+      </c>
+      <c r="T21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>..\data\csvs\nSybxRalRNAi\N1\N1_nSybxRalRNAiBL29580_29C_L3_FA.csv</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>5403</v>
+      </c>
+      <c r="C22" t="n">
+        <v>21.09938922820655</v>
+      </c>
+      <c r="D22" t="n">
+        <v>38</v>
+      </c>
+      <c r="E22" t="n">
+        <v>4</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="n">
+        <v>87.16689580927807</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0.6139955093398315</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0.4743416490252165</v>
+      </c>
+      <c r="K22" t="n">
+        <v>3.891336531321556</v>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>N1</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>nSybxRalRNAi</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>29C_L3_FA</t>
+        </is>
+      </c>
+      <c r="Q22" t="n">
+        <v>0.008951141596460717</v>
+      </c>
+      <c r="R22" t="n">
+        <v>0</v>
+      </c>
+      <c r="S22" t="b">
+        <v>0</v>
+      </c>
+      <c r="T22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>..\data\csvs\nSybxRalRNAi\N1\N1_nSybxRalRNAiBL29580_29C_L4_FA.csv</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>5402</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
+        <v>69.24885158806589</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0.3846446116722786</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0.276586333718905</v>
+      </c>
+      <c r="K23" t="n">
+        <v>7.942241497209713</v>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>N1</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>nSybxRalRNAi</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>29C_L4_FA</t>
+        </is>
+      </c>
+      <c r="Q23" t="n">
+        <v>0.01279888697242738</v>
+      </c>
+      <c r="R23" t="n">
+        <v>0</v>
+      </c>
+      <c r="S23" t="b">
+        <v>0</v>
+      </c>
+      <c r="T23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>..\data\csvs\nSybxRalRNAi\N1\N1_nSybxRalRNAiBL29580_29C_L5_FA.csv</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>5403</v>
+      </c>
+      <c r="C24" t="n">
+        <v>19.23005737553211</v>
+      </c>
+      <c r="D24" t="n">
+        <v>34.63333333333333</v>
+      </c>
+      <c r="E24" t="n">
+        <v>5</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="n">
+        <v>93.82556110788447</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0.6457368279964519</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0.5239274758971829</v>
+      </c>
+      <c r="K24" t="n">
+        <v>3.833079701754197</v>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>N1</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>nSybxRalRNAi</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>29C_L5_FA</t>
+        </is>
+      </c>
+      <c r="Q24" t="n">
+        <v>0.007447800000000282</v>
+      </c>
+      <c r="R24" t="n">
+        <v>0</v>
+      </c>
+      <c r="S24" t="b">
+        <v>0</v>
+      </c>
+      <c r="T24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>..\data\csvs\nSybxRalRNAi\N1\N1_nSybxRalRNAiBL29580_29C_L6_FA.csv</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>5403</v>
+      </c>
+      <c r="C25" t="n">
+        <v>19.78530446048492</v>
+      </c>
+      <c r="D25" t="n">
+        <v>35.63333333333333</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="n">
+        <v>85.3292753092116</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0.5907865818777632</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0.4509988913511996</v>
+      </c>
+      <c r="K25" t="n">
+        <v>3.872208672062936</v>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>N1</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>nSybxRalRNAi</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>29C_L6_FA</t>
+        </is>
+      </c>
+      <c r="Q25" t="n">
+        <v>0.007447800000000282</v>
+      </c>
+      <c r="R25" t="n">
+        <v>0</v>
+      </c>
+      <c r="S25" t="b">
+        <v>0</v>
+      </c>
+      <c r="T25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>..\data\csvs\nSybxRalRNAi\N2\N2_nSybxRalRNAi_L1_FA.csv</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>5402</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
+        <v>17</v>
+      </c>
+      <c r="F26" t="n">
+        <v>17</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="n">
+        <v>143.5257002386665</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0.7972173684799103</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0.6007495318348902</v>
+      </c>
+      <c r="K26" t="n">
+        <v>4.718400152594072</v>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>N2</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>nSybxRalRNAi</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>FA</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="n">
+        <v>0.002482600000011854</v>
+      </c>
+      <c r="R26" t="n">
+        <v>1</v>
+      </c>
+      <c r="S26" t="b">
+        <v>0</v>
+      </c>
+      <c r="T26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>..\data\csvs\nSybxRalRNAi\N2\N2_nSybxRalRNAi_L2_FA.csv</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>5402</v>
+      </c>
+      <c r="C27" t="n">
+        <v>50.0925583117364</v>
+      </c>
+      <c r="D27" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="n">
+        <v>127.869193080765</v>
+      </c>
+      <c r="I27" t="n">
+        <v>1.424461861278481</v>
+      </c>
+      <c r="J27" t="n">
+        <v>1.224132345786134</v>
+      </c>
+      <c r="K27" t="n">
+        <v>5.846383497513595</v>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>N2</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>nSybxRalRNAi</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>FA</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="n">
+        <v>0.007447800000000282</v>
+      </c>
+      <c r="R27" t="n">
+        <v>0</v>
+      </c>
+      <c r="S27" t="b">
+        <v>1</v>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>unusually fast median speed</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>..\data\csvs\nSybxRalRNAi\N2\N2_nSybxRalRNAi_L3_FA.csv</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>5404</v>
+      </c>
+      <c r="C28" t="n">
+        <v>62.76831976313841</v>
+      </c>
+      <c r="D28" t="n">
+        <v>112.5</v>
+      </c>
+      <c r="E28" t="n">
+        <v>13</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" t="n">
+        <v>64.07607585567288</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0.9558837770612564</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0.7648529270386402</v>
+      </c>
+      <c r="K28" t="n">
+        <v>6.413267497929511</v>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>N2</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>nSybxRalRNAi</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>FA</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="n">
+        <v>0.004965199999988428</v>
+      </c>
+      <c r="R28" t="n">
+        <v>0</v>
+      </c>
+      <c r="S28" t="b">
+        <v>0</v>
+      </c>
+      <c r="T28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>..\data\csvs\nSybxRalRNAi\N2\N2_nSybxRalRNAi_L4_FA.csv</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>5402</v>
+      </c>
+      <c r="C29" t="n">
+        <v>31.28470936690115</v>
+      </c>
+      <c r="D29" t="n">
+        <v>46.46666666666667</v>
+      </c>
+      <c r="E29" t="n">
+        <v>64</v>
+      </c>
+      <c r="F29" t="n">
+        <v>36</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="n">
+        <v>121.7477918360766</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0.984748922912456</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0.7874642849043526</v>
+      </c>
+      <c r="K29" t="n">
+        <v>5.368239935025239</v>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>N2</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>nSybxRalRNAi</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>FA</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R29" t="n">
+        <v>2</v>
+      </c>
+      <c r="S29" t="b">
+        <v>0</v>
+      </c>
+      <c r="T29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>..\data\csvs\nSybxRalRNAi\N2\N2_nSybxRalRNAi_L5_FA.csv</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>5402</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" t="n">
+        <v>106.2824328467211</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0.590348636437999</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0.4589117562233681</v>
+      </c>
+      <c r="K30" t="n">
+        <v>4.384928733742462</v>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>N2</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>nSybxRalRNAi</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>L5</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>FA</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="n">
+        <v>0.004965199999997248</v>
+      </c>
+      <c r="R30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S30" t="b">
+        <v>0</v>
+      </c>
+      <c r="T30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>..\data\csvs\nSybxRalRNAi\N2\N2_nSybxRalRNAi_L6_FA.csv</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>5402</v>
+      </c>
+      <c r="C31" t="n">
+        <v>13.90225842280637</v>
+      </c>
+      <c r="D31" t="n">
+        <v>25.03333333333333</v>
+      </c>
+      <c r="E31" t="n">
+        <v>13</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" t="n">
+        <v>120.1010818984415</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0.7750123589918789</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0.6000000000000085</v>
+      </c>
+      <c r="K31" t="n">
+        <v>5.098234988699556</v>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>N2</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>nSybxRalRNAi</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>L6</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>FA</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="n">
+        <v>0.002482599999998624</v>
+      </c>
+      <c r="R31" t="n">
+        <v>0</v>
+      </c>
+      <c r="S31" t="b">
+        <v>0</v>
+      </c>
+      <c r="T31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>..\data\csvs\nSybxRalRNAi\N2\N2_nSybxRalRNAi_L7_FA.csv</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>5402</v>
+      </c>
+      <c r="C32" t="n">
+        <v>54.09107737874861</v>
+      </c>
+      <c r="D32" t="n">
+        <v>97.40000000000001</v>
+      </c>
+      <c r="E32" t="n">
+        <v>113</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" t="n">
+        <v>67.95863427939746</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0.8224118710697556</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0.6007495318351138</v>
+      </c>
+      <c r="K32" t="n">
+        <v>4.158004329002184</v>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>N2</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>nSybxRalRNAi</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>L7</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>FA</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="n">
+        <v>0.002482600000011854</v>
+      </c>
+      <c r="R32" t="n">
+        <v>0</v>
+      </c>
+      <c r="S32" t="b">
+        <v>0</v>
+      </c>
+      <c r="T32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>..\data\csvs\nSybxRalRNAi\N2\N2_nSybxRalRNAi_L8_FA.csv</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>5401</v>
+      </c>
+      <c r="C33" t="n">
+        <v>25.01388631734864</v>
+      </c>
+      <c r="D33" t="n">
+        <v>45.03333333333333</v>
+      </c>
+      <c r="E33" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" t="n">
+        <v>111.3886815264712</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0.825509003407642</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0.61846584384272</v>
+      </c>
+      <c r="K33" t="n">
+        <v>4.272762572388041</v>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>N2</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>nSybxRalRNAi</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>L8</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>FA</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="n">
+        <v>0.004965199999988428</v>
+      </c>
+      <c r="R33" t="n">
+        <v>0</v>
+      </c>
+      <c r="S33" t="b">
+        <v>0</v>
+      </c>
+      <c r="T33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>..\data\csvs\nSybxRalRNAi\N2\N2_nSybxRalRNAi_L9_FA.csv</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>5402</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0.1666666666666667</v>
+      </c>
+      <c r="E34" t="n">
+        <v>5</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" t="n">
+        <v>94.57955518017006</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0.5258314780217016</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0.4013710789368652</v>
+      </c>
+      <c r="K34" t="n">
+        <v>3.294267748681114</v>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>N2</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>nSybxRalRNAi</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>L9</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>FA</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr"/>
+      <c r="Q34" t="n">
+        <v>0.007447800000000282</v>
+      </c>
+      <c r="R34" t="n">
+        <v>0</v>
+      </c>
+      <c r="S34" t="b">
+        <v>0</v>
+      </c>
+      <c r="T34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>..\data\csvs\nSybxRalRNAi\N3\N3_nSybxRalRNAi_L1_FA.csv</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>5402</v>
+      </c>
+      <c r="C35" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" t="n">
+        <v>87.21447328052088</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0.4844351413470888</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0.3710795063056035</v>
+      </c>
+      <c r="K35" t="n">
+        <v>3.142133033466354</v>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>N3</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>nSybxRalRNAi</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>FA</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="n">
+        <v>0.007447800000000282</v>
+      </c>
+      <c r="R35" t="n">
+        <v>0</v>
+      </c>
+      <c r="S35" t="b">
+        <v>0</v>
+      </c>
+      <c r="T35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>..\data\csvs\nSybxRalRNAi\N3\N3_nSybxRalRNAi_L2_FA.csv</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>5402</v>
+      </c>
+      <c r="C36" t="n">
+        <v>27.78600518326546</v>
+      </c>
+      <c r="D36" t="n">
+        <v>50.03333333333333</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" t="n">
+        <v>72.04662166194157</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0.5542047820149353</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0.4242640687118441</v>
+      </c>
+      <c r="K36" t="n">
+        <v>3.012573650552031</v>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>N3</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>nSybxRalRNAi</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>FA</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr"/>
+      <c r="Q36" t="n">
+        <v>0.007021853179890999</v>
+      </c>
+      <c r="R36" t="n">
+        <v>0</v>
+      </c>
+      <c r="S36" t="b">
+        <v>0</v>
+      </c>
+      <c r="T36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>..\data\csvs\nSybxRalRNAi\N3\N3_nSybxRalRNAi_L3_FA.csv</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>5402</v>
+      </c>
+      <c r="C37" t="n">
+        <v>38.68937430581266</v>
+      </c>
+      <c r="D37" t="n">
+        <v>52.16666666666666</v>
+      </c>
+      <c r="E37" t="n">
+        <v>43</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" t="n">
+        <v>68.68420079634333</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0.6227035430312178</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0.4459820624195625</v>
+      </c>
+      <c r="K37" t="n">
+        <v>3.947708195903186</v>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>N3</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>nSybxRalRNAi</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>FA</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="n">
+        <v>0.004965200000023708</v>
+      </c>
+      <c r="R37" t="n">
+        <v>0</v>
+      </c>
+      <c r="S37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T37" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>